<commit_message>
added backend and frontend
</commit_message>
<xml_diff>
--- a/docs/System_Test_Report_template.xlsx
+++ b/docs/System_Test_Report_template.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D588E4AF-5D52-4F16-844F-97239BBD583C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Test Report" sheetId="2" r:id="rId1"/>
     <sheet name="Test Cases &amp; Results" sheetId="1" r:id="rId2"/>
     <sheet name="Enums" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -20,6 +21,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -101,7 +104,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -229,14 +232,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -248,13 +244,6 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -311,7 +300,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1208,9 +1196,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1248,9 +1236,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1285,7 +1273,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1320,7 +1308,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1493,14 +1481,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:C6"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1509,7 +1497,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -1518,7 +1506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
@@ -1527,7 +1515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>3</v>
       </c>
@@ -1544,23 +1532,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:K22"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="28.140625" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" customWidth="1"/>
-    <col min="8" max="8" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" customWidth="1"/>
-    <col min="10" max="10" width="18.5703125" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="28.109375" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
+    <col min="8" max="8" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1592,7 +1580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -1624,7 +1612,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B4" s="2">
         <f>B3+1</f>
         <v>2</v>
@@ -1641,7 +1629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="2">
         <f t="shared" ref="B5:B20" si="0">B4+1</f>
         <v>3</v>
@@ -1658,7 +1646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1675,7 +1663,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1692,7 +1680,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1709,7 +1697,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1726,7 +1714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B10" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1743,7 +1731,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B11" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1760,7 +1748,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B12" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1777,7 +1765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B13" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1794,7 +1782,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B14" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1811,7 +1799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B15" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1828,7 +1816,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B16" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1845,7 +1833,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B17" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1862,7 +1850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B18" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1879,7 +1867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B19" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1896,7 +1884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B20" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1913,7 +1901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B21" s="2">
         <f t="shared" ref="B21:B22" si="1">B20+1</f>
         <v>19</v>
@@ -1930,7 +1918,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B22" s="2">
         <f t="shared" si="1"/>
         <v>20</v>
@@ -1948,24 +1936,12 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K3:K20">
-    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
-      <formula>"Fail"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:K20">
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+  <conditionalFormatting sqref="K3:K22">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Not Tested"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K21:K22">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Fail"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K21:K22">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Not Tested"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1973,13 +1949,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
             <xm:f>Enums!$B$8:$B$10</xm:f>
           </x14:formula1>
           <xm:sqref>E3:E5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
             <xm:f>Enums!$B$2:$B$4</xm:f>
           </x14:formula1>
@@ -1992,36 +1968,36 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:B10"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>17</v>
       </c>
@@ -2033,21 +2009,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E81D8C8DDAE8BD44A422697963F06C45" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b6816e004dbb89c674e51f5647972552">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2b02348f-b4e3-458c-83fc-9e90db0f8029" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e6418ca14ac9ee17b8bbf6df78e0c223" ns2:_="">
     <xsd:import namespace="2b02348f-b4e3-458c-83fc-9e90db0f8029"/>
@@ -2205,31 +2166,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69DB72C7-DF0B-4E18-8174-00AB852E6FB4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2b02348f-b4e3-458c-83fc-9e90db0f8029"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{859B513B-8BED-4B59-B224-E0A2C6173D25}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCDB6385-31B2-4574-9AA4-BF13B563A4E3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2245,4 +2197,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{859B513B-8BED-4B59-B224-E0A2C6173D25}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69DB72C7-DF0B-4E18-8174-00AB852E6FB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2b02348f-b4e3-458c-83fc-9e90db0f8029"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>